<commit_message>
Clean up project, fix PPS bugs, add keep-alive, update config
- Archive 37 docs, 14 generator scripts, orphaned pages to _archive/
- Fix PPS page crash (wrong save_pps_survey arg order + validator return type)
- Fix PPS gauge color visibility (dark containers for chart readability)
- Fix db.py Yes/No text handling for PPS boolean fields
- Add keep-alive JS ping (2min interval) to prevent session timeout
- Update .streamlit/config.toml (CORS, websocket, headless, fastReruns)
- Update .gitignore: track .streamlit/, exclude _archive/
- Remove orphaned pages (page_gass, page_env_surveillance, page_public)
- Add new modules: alerts, antibiogram, scheduler, whonet, validate_onehealth
- Add One Health PPS/AMU/AMC dashboard pages
- Add data lookups and KoboToolbox config
</commit_message>
<xml_diff>
--- a/templates/AMR_ENV_FOOD_template_v1.xlsx
+++ b/templates/AMR_ENV_FOOD_template_v1.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="samples" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ast_results" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="samples" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ast_results" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lab_lists" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,50 +438,55 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>lab_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>collection_date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>region</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>district</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>site_type</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>source_category</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>source_type</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>food_matrix</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>environment_matrix</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>latitude</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>longitude</t>
         </is>
@@ -494,44 +500,48 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Accra Veterinary Laboratory</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>2024-01-15</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Ashanti</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Kumasi</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Water Treatment</t>
-        </is>
-      </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>Water Treatment Plant</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>ENVIRONMENT</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>water</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>treated_water</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>treated_water</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
         <v>6.6326</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>-1.6243</v>
       </c>
     </row>
@@ -543,48 +553,105 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Alma Medical Laboratory Ltd</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>2024-01-20</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Greater Accra</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Accra</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Farm</t>
-        </is>
-      </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>Retail Market</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>FOOD</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>meat</t>
-        </is>
-      </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>raw_chicken</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>chicken</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>5.6037</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>-0.187</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SAMPLE_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CSIR – Water Research Institute (Microbiology Laboratory)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2024-01-25</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Eastern</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Koforidua</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Hospital Lab</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>HUMAN</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>clinical_specimen</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>6.1256</v>
+      </c>
+      <c r="L4" t="n">
+        <v>-0.3597</v>
+      </c>
+    </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>lab_lists!$A$2:$A$20</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -595,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -644,6 +711,11 @@
           <t>mic_value</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>zone_diameter</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -686,7 +758,9 @@
           <t>2024-01-20</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -729,7 +803,9 @@
           <t>2024-01-20</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -774,6 +850,160 @@
       </c>
       <c r="I4" t="n">
         <v>0.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>lab_name_list</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Accra Veterinary Laboratory</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Alma Medical Laboratory Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CSIR – Water Research Institute (Microbiology Laboratory)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cape Coast Teaching Hospital</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Central Veterinary Laboratory</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Eastern Regional Hospital</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ho Teaching Hospital</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Komfo Anokye Teaching Hospital</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Korle-Bu Teaching Hospital</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Kumasi Veterinary Laboratory</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Lekma Hospital</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Metropolis Health Care Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>National Food Safety Laboratory</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Pong Tamale School</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Quadushah Medical Diagnostic Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sekondi Public Health Reference Laboratory</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>St. Martin De Porres Hospital Eikwe</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Sunyani Teaching Hospital</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Tamale Teaching Hospital</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>